<commit_message>
fixed PG conn and add secret data to products.csv
</commit_message>
<xml_diff>
--- a/code/backend/data/raw/products.xlsx
+++ b/code/backend/data/raw/products.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/b8827725017ffd42/Documents/GitHub/GROUP_10_TOPIC_10_SEMANTIC_SEARCH/backend/data/raw/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/b8827725017ffd42/Documents/GitHub/GROUP_10_TOPIC_10_SEMANTIC_SEARCH/code/backend/data/raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{667693E6-60E9-475C-B20E-C088DDFF364E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{12B4B746-46F8-4778-ADFC-4DBC66A08956}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{667693E6-60E9-475C-B20E-C088DDFF364E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B99C6739-1512-4F20-A883-31D5EB182DB4}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="3324" yWindow="2604" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1247,36 +1247,6 @@
     <t>"Siêu phẩm đời đầu" nhưng chưa bao giờ lỗi mốt. Đây là mẫu máy bay mà chính phủ Mỹ ích kỷ đến mức cấm xuất khẩu cho bất kỳ ai. Nó tàng hình tốt đến mức radar đối phương thường nhầm nó với một con chim sẻ đang bay ở vận tốc siêu thanh.</t>
   </si>
   <si>
-    <t>stealth aircraft/stealthAircraft_10.jpg</t>
-  </si>
-  <si>
-    <t>stealth aircraft/stealthAircraft_01.jpg</t>
-  </si>
-  <si>
-    <t>stealth aircraft/stealthAircraft_02.jpg</t>
-  </si>
-  <si>
-    <t>stealth aircraft/stealthAircraft_03.jpg</t>
-  </si>
-  <si>
-    <t>stealth aircraft/stealthAircraft_04.jpg</t>
-  </si>
-  <si>
-    <t>stealth aircraft/stealthAircraft_05.jpg</t>
-  </si>
-  <si>
-    <t>stealth aircraft/stealthAircraft_06.jpg</t>
-  </si>
-  <si>
-    <t>stealth aircraft/stealthAircraft_09.jpg</t>
-  </si>
-  <si>
-    <t>stealth aircraft/stealthAircraft_08.jpg</t>
-  </si>
-  <si>
-    <t>stealth aircraft/stealthAircraft_07.jpg</t>
-  </si>
-  <si>
     <t>Chiếc "iPhone" của giới không quân. Nó đầy rẫy công nghệ và phần mềm phức tạp, đôi khi gặp lỗi cập nhật (bug), nhưng một khi đã chạy mượt thì nó sẽ kết nối mọi thứ trên chiến trường vào màn hình của phi công như chơi game.</t>
   </si>
   <si>
@@ -1605,6 +1575,36 @@
   </si>
   <si>
     <t>president/president_1.jpg</t>
+  </si>
+  <si>
+    <t>stealthAircraft/stealthAircraft_01.jpg</t>
+  </si>
+  <si>
+    <t>stealthAircraft/stealthAircraft_02.jpg</t>
+  </si>
+  <si>
+    <t>stealthAircraft/stealthAircraft_03.jpg</t>
+  </si>
+  <si>
+    <t>stealthAircraft/stealthAircraft_04.jpg</t>
+  </si>
+  <si>
+    <t>stealthAircraft/stealthAircraft_05.jpg</t>
+  </si>
+  <si>
+    <t>stealthAircraft/stealthAircraft_06.jpg</t>
+  </si>
+  <si>
+    <t>stealthAircraft/stealthAircraft_07.jpg</t>
+  </si>
+  <si>
+    <t>stealthAircraft/stealthAircraft_08.jpg</t>
+  </si>
+  <si>
+    <t>stealthAircraft/stealthAircraft_09.jpg</t>
+  </si>
+  <si>
+    <t>stealthAircraft/stealthAircraft_10.jpg</t>
   </si>
 </sst>
 </file>
@@ -1675,6 +1675,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4290,7 +4294,7 @@
         <v>640000</v>
       </c>
       <c r="F102" s="1" t="s">
-        <v>512</v>
+        <v>502</v>
       </c>
       <c r="G102" s="1" t="s">
         <v>377</v>
@@ -4313,7 +4317,7 @@
         <v>630000</v>
       </c>
       <c r="F103" s="1" t="s">
-        <v>512</v>
+        <v>502</v>
       </c>
       <c r="G103" s="1" t="s">
         <v>378</v>
@@ -4336,7 +4340,7 @@
         <v>347000</v>
       </c>
       <c r="F104" s="1" t="s">
-        <v>512</v>
+        <v>502</v>
       </c>
       <c r="G104" s="1" t="s">
         <v>379</v>
@@ -4359,7 +4363,7 @@
         <v>138000</v>
       </c>
       <c r="F105" s="1" t="s">
-        <v>512</v>
+        <v>502</v>
       </c>
       <c r="G105" s="1" t="s">
         <v>380</v>
@@ -4382,7 +4386,7 @@
         <v>1750000</v>
       </c>
       <c r="F106" s="1" t="s">
-        <v>512</v>
+        <v>502</v>
       </c>
       <c r="G106" s="1" t="s">
         <v>381</v>
@@ -4405,7 +4409,7 @@
         <v>360000</v>
       </c>
       <c r="F107" s="1" t="s">
-        <v>512</v>
+        <v>502</v>
       </c>
       <c r="G107" s="1" t="s">
         <v>382</v>
@@ -4428,7 +4432,7 @@
         <v>827500</v>
       </c>
       <c r="F108" s="1" t="s">
-        <v>512</v>
+        <v>502</v>
       </c>
       <c r="G108" s="1" t="s">
         <v>383</v>
@@ -4451,7 +4455,7 @@
         <v>8960000</v>
       </c>
       <c r="F109" s="1" t="s">
-        <v>512</v>
+        <v>502</v>
       </c>
       <c r="G109" s="1" t="s">
         <v>384</v>
@@ -4474,7 +4478,7 @@
         <v>318000</v>
       </c>
       <c r="F110" s="1" t="s">
-        <v>512</v>
+        <v>502</v>
       </c>
       <c r="G110" s="1" t="s">
         <v>385</v>
@@ -4497,7 +4501,7 @@
         <v>827000</v>
       </c>
       <c r="F111" s="1" t="s">
-        <v>512</v>
+        <v>502</v>
       </c>
       <c r="G111" s="1" t="s">
         <v>386</v>
@@ -4520,7 +4524,7 @@
         <v>350000</v>
       </c>
       <c r="F112" s="1" t="s">
-        <v>394</v>
+        <v>503</v>
       </c>
       <c r="G112" s="1" t="s">
         <v>392</v>
@@ -4543,10 +4547,10 @@
         <v>110000</v>
       </c>
       <c r="F113" s="1" t="s">
-        <v>395</v>
+        <v>504</v>
       </c>
       <c r="G113" s="1" t="s">
-        <v>403</v>
+        <v>393</v>
       </c>
     </row>
     <row r="114" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
@@ -4566,10 +4570,10 @@
         <v>50000</v>
       </c>
       <c r="F114" s="1" t="s">
-        <v>396</v>
+        <v>505</v>
       </c>
       <c r="G114" s="1" t="s">
-        <v>404</v>
+        <v>394</v>
       </c>
     </row>
     <row r="115" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
@@ -4589,10 +4593,10 @@
         <v>120000</v>
       </c>
       <c r="F115" s="1" t="s">
-        <v>397</v>
+        <v>506</v>
       </c>
       <c r="G115" s="1" t="s">
-        <v>405</v>
+        <v>395</v>
       </c>
     </row>
     <row r="116" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
@@ -4612,10 +4616,10 @@
         <v>2100000</v>
       </c>
       <c r="F116" s="1" t="s">
-        <v>398</v>
+        <v>507</v>
       </c>
       <c r="G116" s="1" t="s">
-        <v>406</v>
+        <v>396</v>
       </c>
     </row>
     <row r="117" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
@@ -4626,7 +4630,7 @@
         <v>2</v>
       </c>
       <c r="C117" s="1" t="s">
-        <v>407</v>
+        <v>397</v>
       </c>
       <c r="D117" s="1" t="s">
         <v>372</v>
@@ -4635,10 +4639,10 @@
         <v>750000</v>
       </c>
       <c r="F117" s="1" t="s">
-        <v>399</v>
+        <v>508</v>
       </c>
       <c r="G117" s="1" t="s">
-        <v>408</v>
+        <v>398</v>
       </c>
     </row>
     <row r="118" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
@@ -4649,7 +4653,7 @@
         <v>2</v>
       </c>
       <c r="C118" s="1" t="s">
-        <v>409</v>
+        <v>399</v>
       </c>
       <c r="D118" s="1" t="s">
         <v>365</v>
@@ -4658,10 +4662,10 @@
         <v>80000</v>
       </c>
       <c r="F118" s="1" t="s">
-        <v>402</v>
+        <v>509</v>
       </c>
       <c r="G118" s="1" t="s">
-        <v>410</v>
+        <v>400</v>
       </c>
     </row>
     <row r="119" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
@@ -4672,7 +4676,7 @@
         <v>2</v>
       </c>
       <c r="C119" s="1" t="s">
-        <v>411</v>
+        <v>401</v>
       </c>
       <c r="D119" s="1" t="s">
         <v>367</v>
@@ -4681,10 +4685,10 @@
         <v>100000</v>
       </c>
       <c r="F119" s="1" t="s">
-        <v>401</v>
+        <v>510</v>
       </c>
       <c r="G119" s="1" t="s">
-        <v>412</v>
+        <v>402</v>
       </c>
     </row>
     <row r="120" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
@@ -4695,19 +4699,19 @@
         <v>2</v>
       </c>
       <c r="C120" s="1" t="s">
-        <v>413</v>
+        <v>403</v>
       </c>
       <c r="D120" s="1" t="s">
-        <v>416</v>
+        <v>406</v>
       </c>
       <c r="E120" s="1">
         <v>100000</v>
       </c>
       <c r="F120" s="1" t="s">
-        <v>400</v>
+        <v>511</v>
       </c>
       <c r="G120" s="1" t="s">
-        <v>414</v>
+        <v>404</v>
       </c>
     </row>
     <row r="121" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
@@ -4718,7 +4722,7 @@
         <v>2</v>
       </c>
       <c r="C121" s="1" t="s">
-        <v>415</v>
+        <v>405</v>
       </c>
       <c r="D121" s="1" t="s">
         <v>372</v>
@@ -4727,10 +4731,10 @@
         <v>111000</v>
       </c>
       <c r="F121" s="1" t="s">
-        <v>393</v>
+        <v>512</v>
       </c>
       <c r="G121" s="1" t="s">
-        <v>417</v>
+        <v>407</v>
       </c>
     </row>
     <row r="122" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
@@ -4741,7 +4745,7 @@
         <v>2</v>
       </c>
       <c r="C122" s="1" t="s">
-        <v>418</v>
+        <v>408</v>
       </c>
       <c r="D122" s="1" t="s">
         <v>372</v>
@@ -4750,10 +4754,10 @@
         <v>200000</v>
       </c>
       <c r="F122" s="1" t="s">
-        <v>438</v>
+        <v>428</v>
       </c>
       <c r="G122" s="1" t="s">
-        <v>419</v>
+        <v>409</v>
       </c>
     </row>
     <row r="123" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
@@ -4764,7 +4768,7 @@
         <v>2</v>
       </c>
       <c r="C123" s="1" t="s">
-        <v>420</v>
+        <v>410</v>
       </c>
       <c r="D123" s="1" t="s">
         <v>372</v>
@@ -4773,10 +4777,10 @@
         <v>200000</v>
       </c>
       <c r="F123" s="1" t="s">
-        <v>439</v>
+        <v>429</v>
       </c>
       <c r="G123" s="1" t="s">
-        <v>421</v>
+        <v>411</v>
       </c>
     </row>
     <row r="124" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
@@ -4787,7 +4791,7 @@
         <v>2</v>
       </c>
       <c r="C124" s="1" t="s">
-        <v>422</v>
+        <v>412</v>
       </c>
       <c r="D124" s="1" t="s">
         <v>366</v>
@@ -4796,10 +4800,10 @@
         <v>150000</v>
       </c>
       <c r="F124" s="1" t="s">
-        <v>440</v>
+        <v>430</v>
       </c>
       <c r="G124" s="1" t="s">
-        <v>423</v>
+        <v>413</v>
       </c>
     </row>
     <row r="125" spans="1:7" ht="72" x14ac:dyDescent="0.3">
@@ -4810,7 +4814,7 @@
         <v>2</v>
       </c>
       <c r="C125" s="1" t="s">
-        <v>424</v>
+        <v>414</v>
       </c>
       <c r="D125" s="1" t="s">
         <v>372</v>
@@ -4819,10 +4823,10 @@
         <v>28000</v>
       </c>
       <c r="F125" s="1" t="s">
-        <v>441</v>
+        <v>431</v>
       </c>
       <c r="G125" s="1" t="s">
-        <v>436</v>
+        <v>426</v>
       </c>
     </row>
     <row r="126" spans="1:7" ht="86.4" x14ac:dyDescent="0.3">
@@ -4833,7 +4837,7 @@
         <v>2</v>
       </c>
       <c r="C126" s="1" t="s">
-        <v>425</v>
+        <v>415</v>
       </c>
       <c r="D126" s="1" t="s">
         <v>372</v>
@@ -4842,10 +4846,10 @@
         <v>25000</v>
       </c>
       <c r="F126" s="1" t="s">
-        <v>442</v>
+        <v>432</v>
       </c>
       <c r="G126" s="1" t="s">
-        <v>437</v>
+        <v>427</v>
       </c>
     </row>
     <row r="127" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
@@ -4856,7 +4860,7 @@
         <v>2</v>
       </c>
       <c r="C127" s="1" t="s">
-        <v>426</v>
+        <v>416</v>
       </c>
       <c r="D127" s="1" t="s">
         <v>366</v>
@@ -4865,10 +4869,10 @@
         <v>150000</v>
       </c>
       <c r="F127" s="1" t="s">
-        <v>443</v>
+        <v>433</v>
       </c>
       <c r="G127" s="1" t="s">
-        <v>427</v>
+        <v>417</v>
       </c>
     </row>
     <row r="128" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
@@ -4879,7 +4883,7 @@
         <v>2</v>
       </c>
       <c r="C128" s="1" t="s">
-        <v>428</v>
+        <v>418</v>
       </c>
       <c r="D128" s="1" t="s">
         <v>366</v>
@@ -4888,10 +4892,10 @@
         <v>150000</v>
       </c>
       <c r="F128" s="1" t="s">
-        <v>444</v>
+        <v>434</v>
       </c>
       <c r="G128" s="1" t="s">
-        <v>429</v>
+        <v>419</v>
       </c>
     </row>
     <row r="129" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
@@ -4902,7 +4906,7 @@
         <v>2</v>
       </c>
       <c r="C129" s="1" t="s">
-        <v>430</v>
+        <v>420</v>
       </c>
       <c r="D129" s="1" t="s">
         <v>365</v>
@@ -4911,10 +4915,10 @@
         <v>150000</v>
       </c>
       <c r="F129" s="1" t="s">
-        <v>445</v>
+        <v>435</v>
       </c>
       <c r="G129" s="1" t="s">
-        <v>431</v>
+        <v>421</v>
       </c>
     </row>
     <row r="130" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
@@ -4925,7 +4929,7 @@
         <v>2</v>
       </c>
       <c r="C130" s="1" t="s">
-        <v>432</v>
+        <v>422</v>
       </c>
       <c r="D130" s="1" t="s">
         <v>372</v>
@@ -4934,10 +4938,10 @@
         <v>70000</v>
       </c>
       <c r="F130" s="1" t="s">
-        <v>446</v>
+        <v>436</v>
       </c>
       <c r="G130" s="1" t="s">
-        <v>433</v>
+        <v>423</v>
       </c>
     </row>
     <row r="131" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
@@ -4948,7 +4952,7 @@
         <v>2</v>
       </c>
       <c r="C131" s="1" t="s">
-        <v>434</v>
+        <v>424</v>
       </c>
       <c r="D131" s="1" t="s">
         <v>372</v>
@@ -4957,10 +4961,10 @@
         <v>31000</v>
       </c>
       <c r="F131" s="1" t="s">
-        <v>447</v>
+        <v>437</v>
       </c>
       <c r="G131" s="1" t="s">
-        <v>435</v>
+        <v>425</v>
       </c>
     </row>
     <row r="132" spans="1:7" ht="72" x14ac:dyDescent="0.3">
@@ -4971,7 +4975,7 @@
         <v>1</v>
       </c>
       <c r="C132" s="1" t="s">
-        <v>448</v>
+        <v>438</v>
       </c>
       <c r="D132" s="1" t="s">
         <v>366</v>
@@ -4980,10 +4984,10 @@
         <v>1200</v>
       </c>
       <c r="F132" s="1" t="s">
+        <v>439</v>
+      </c>
+      <c r="G132" s="1" t="s">
         <v>449</v>
-      </c>
-      <c r="G132" s="1" t="s">
-        <v>459</v>
       </c>
     </row>
     <row r="133" spans="1:7" ht="72" x14ac:dyDescent="0.3">
@@ -4994,7 +4998,7 @@
         <v>1</v>
       </c>
       <c r="C133" s="1" t="s">
-        <v>460</v>
+        <v>450</v>
       </c>
       <c r="D133" s="1" t="s">
         <v>372</v>
@@ -5003,10 +5007,10 @@
         <v>1500</v>
       </c>
       <c r="F133" s="1" t="s">
-        <v>450</v>
+        <v>440</v>
       </c>
       <c r="G133" s="1" t="s">
-        <v>461</v>
+        <v>451</v>
       </c>
     </row>
     <row r="134" spans="1:7" ht="72" x14ac:dyDescent="0.3">
@@ -5017,7 +5021,7 @@
         <v>1</v>
       </c>
       <c r="C134" s="1" t="s">
-        <v>462</v>
+        <v>452</v>
       </c>
       <c r="D134" s="1" t="s">
         <v>372</v>
@@ -5026,10 +5030,10 @@
         <v>2500</v>
       </c>
       <c r="F134" s="1" t="s">
-        <v>451</v>
+        <v>441</v>
       </c>
       <c r="G134" s="1" t="s">
-        <v>463</v>
+        <v>453</v>
       </c>
     </row>
     <row r="135" spans="1:7" ht="72" x14ac:dyDescent="0.3">
@@ -5040,19 +5044,19 @@
         <v>1</v>
       </c>
       <c r="C135" s="1" t="s">
-        <v>464</v>
+        <v>454</v>
       </c>
       <c r="D135" s="1" t="s">
-        <v>465</v>
+        <v>455</v>
       </c>
       <c r="E135" s="1">
         <v>550</v>
       </c>
       <c r="F135" s="1" t="s">
-        <v>452</v>
+        <v>442</v>
       </c>
       <c r="G135" s="1" t="s">
-        <v>466</v>
+        <v>456</v>
       </c>
     </row>
     <row r="136" spans="1:7" ht="72" x14ac:dyDescent="0.3">
@@ -5063,7 +5067,7 @@
         <v>1</v>
       </c>
       <c r="C136" s="1" t="s">
-        <v>467</v>
+        <v>457</v>
       </c>
       <c r="D136" s="1" t="s">
         <v>372</v>
@@ -5072,10 +5076,10 @@
         <v>1000</v>
       </c>
       <c r="F136" s="1" t="s">
-        <v>453</v>
+        <v>443</v>
       </c>
       <c r="G136" s="1" t="s">
-        <v>468</v>
+        <v>458</v>
       </c>
     </row>
     <row r="137" spans="1:7" ht="72" x14ac:dyDescent="0.3">
@@ -5086,19 +5090,19 @@
         <v>1</v>
       </c>
       <c r="C137" s="1" t="s">
-        <v>469</v>
+        <v>459</v>
       </c>
       <c r="D137" s="1" t="s">
-        <v>470</v>
+        <v>460</v>
       </c>
       <c r="E137" s="1">
         <v>3000</v>
       </c>
       <c r="F137" s="1" t="s">
-        <v>454</v>
+        <v>444</v>
       </c>
       <c r="G137" s="1" t="s">
-        <v>471</v>
+        <v>461</v>
       </c>
     </row>
     <row r="138" spans="1:7" ht="72" x14ac:dyDescent="0.3">
@@ -5109,7 +5113,7 @@
         <v>1</v>
       </c>
       <c r="C138" s="1" t="s">
-        <v>472</v>
+        <v>462</v>
       </c>
       <c r="D138" s="1" t="s">
         <v>372</v>
@@ -5118,10 +5122,10 @@
         <v>1200</v>
       </c>
       <c r="F138" s="1" t="s">
-        <v>455</v>
+        <v>445</v>
       </c>
       <c r="G138" s="1" t="s">
-        <v>473</v>
+        <v>463</v>
       </c>
     </row>
     <row r="139" spans="1:7" ht="72" x14ac:dyDescent="0.3">
@@ -5132,19 +5136,19 @@
         <v>1</v>
       </c>
       <c r="C139" s="1" t="s">
-        <v>474</v>
+        <v>464</v>
       </c>
       <c r="D139" s="1" t="s">
-        <v>475</v>
+        <v>465</v>
       </c>
       <c r="E139" s="1">
         <v>2300</v>
       </c>
       <c r="F139" s="1" t="s">
-        <v>456</v>
+        <v>446</v>
       </c>
       <c r="G139" s="1" t="s">
-        <v>476</v>
+        <v>466</v>
       </c>
     </row>
     <row r="140" spans="1:7" ht="72" x14ac:dyDescent="0.3">
@@ -5155,7 +5159,7 @@
         <v>1</v>
       </c>
       <c r="C140" s="1" t="s">
-        <v>477</v>
+        <v>467</v>
       </c>
       <c r="D140" s="1" t="s">
         <v>366</v>
@@ -5164,10 +5168,10 @@
         <v>6000</v>
       </c>
       <c r="F140" s="1" t="s">
-        <v>457</v>
+        <v>447</v>
       </c>
       <c r="G140" s="1" t="s">
-        <v>478</v>
+        <v>468</v>
       </c>
     </row>
     <row r="141" spans="1:7" ht="72" x14ac:dyDescent="0.3">
@@ -5178,7 +5182,7 @@
         <v>1</v>
       </c>
       <c r="C141" s="1" t="s">
-        <v>479</v>
+        <v>469</v>
       </c>
       <c r="D141" s="1" t="s">
         <v>372</v>
@@ -5187,10 +5191,10 @@
         <v>500</v>
       </c>
       <c r="F141" s="1" t="s">
-        <v>458</v>
+        <v>448</v>
       </c>
       <c r="G141" s="1" t="s">
-        <v>480</v>
+        <v>470</v>
       </c>
     </row>
     <row r="142" spans="1:7" ht="86.4" x14ac:dyDescent="0.3">
@@ -5201,7 +5205,7 @@
         <v>1</v>
       </c>
       <c r="C142" s="1" t="s">
-        <v>481</v>
+        <v>471</v>
       </c>
       <c r="D142" s="1" t="s">
         <v>372</v>
@@ -5210,10 +5214,10 @@
         <v>2500</v>
       </c>
       <c r="F142" s="1" t="s">
-        <v>502</v>
+        <v>492</v>
       </c>
       <c r="G142" s="1" t="s">
-        <v>482</v>
+        <v>472</v>
       </c>
     </row>
     <row r="143" spans="1:7" ht="72" x14ac:dyDescent="0.3">
@@ -5224,7 +5228,7 @@
         <v>1</v>
       </c>
       <c r="C143" s="1" t="s">
-        <v>483</v>
+        <v>473</v>
       </c>
       <c r="D143" s="1" t="s">
         <v>366</v>
@@ -5233,10 +5237,10 @@
         <v>2000</v>
       </c>
       <c r="F143" s="1" t="s">
-        <v>511</v>
+        <v>501</v>
       </c>
       <c r="G143" s="1" t="s">
-        <v>484</v>
+        <v>474</v>
       </c>
     </row>
     <row r="144" spans="1:7" ht="86.4" x14ac:dyDescent="0.3">
@@ -5247,7 +5251,7 @@
         <v>1</v>
       </c>
       <c r="C144" s="1" t="s">
-        <v>485</v>
+        <v>475</v>
       </c>
       <c r="D144" s="1" t="s">
         <v>372</v>
@@ -5256,10 +5260,10 @@
         <v>25000</v>
       </c>
       <c r="F144" s="1" t="s">
-        <v>510</v>
+        <v>500</v>
       </c>
       <c r="G144" s="1" t="s">
-        <v>486</v>
+        <v>476</v>
       </c>
     </row>
     <row r="145" spans="1:7" ht="72" x14ac:dyDescent="0.3">
@@ -5270,19 +5274,19 @@
         <v>1</v>
       </c>
       <c r="C145" s="1" t="s">
-        <v>487</v>
+        <v>477</v>
       </c>
       <c r="D145" s="1" t="s">
-        <v>488</v>
+        <v>478</v>
       </c>
       <c r="E145" s="1">
         <v>20000</v>
       </c>
       <c r="F145" s="1" t="s">
-        <v>509</v>
+        <v>499</v>
       </c>
       <c r="G145" s="1" t="s">
-        <v>489</v>
+        <v>479</v>
       </c>
     </row>
     <row r="146" spans="1:7" ht="72" x14ac:dyDescent="0.3">
@@ -5293,19 +5297,19 @@
         <v>1</v>
       </c>
       <c r="C146" s="1" t="s">
-        <v>490</v>
+        <v>480</v>
       </c>
       <c r="D146" s="1" t="s">
-        <v>470</v>
+        <v>460</v>
       </c>
       <c r="E146" s="1">
         <v>10000</v>
       </c>
       <c r="F146" s="1" t="s">
-        <v>508</v>
+        <v>498</v>
       </c>
       <c r="G146" s="1" t="s">
-        <v>491</v>
+        <v>481</v>
       </c>
     </row>
     <row r="147" spans="1:7" ht="72" x14ac:dyDescent="0.3">
@@ -5316,19 +5320,19 @@
         <v>1</v>
       </c>
       <c r="C147" s="1" t="s">
-        <v>492</v>
+        <v>482</v>
       </c>
       <c r="D147" s="1" t="s">
-        <v>488</v>
+        <v>478</v>
       </c>
       <c r="E147" s="1">
         <v>2500</v>
       </c>
       <c r="F147" s="1" t="s">
-        <v>507</v>
+        <v>497</v>
       </c>
       <c r="G147" s="1" t="s">
-        <v>493</v>
+        <v>483</v>
       </c>
     </row>
     <row r="148" spans="1:7" ht="72" x14ac:dyDescent="0.3">
@@ -5339,7 +5343,7 @@
         <v>1</v>
       </c>
       <c r="C148" s="1" t="s">
-        <v>494</v>
+        <v>484</v>
       </c>
       <c r="D148" s="1" t="s">
         <v>372</v>
@@ -5348,10 +5352,10 @@
         <v>2000</v>
       </c>
       <c r="F148" s="1" t="s">
-        <v>506</v>
+        <v>496</v>
       </c>
       <c r="G148" s="1" t="s">
-        <v>495</v>
+        <v>485</v>
       </c>
     </row>
     <row r="149" spans="1:7" ht="72" x14ac:dyDescent="0.3">
@@ -5362,7 +5366,7 @@
         <v>1</v>
       </c>
       <c r="C149" s="1" t="s">
-        <v>496</v>
+        <v>486</v>
       </c>
       <c r="D149" s="1" t="s">
         <v>372</v>
@@ -5371,10 +5375,10 @@
         <v>50000</v>
       </c>
       <c r="F149" s="1" t="s">
-        <v>505</v>
+        <v>495</v>
       </c>
       <c r="G149" s="1" t="s">
-        <v>497</v>
+        <v>487</v>
       </c>
     </row>
     <row r="150" spans="1:7" ht="72" x14ac:dyDescent="0.3">
@@ -5385,7 +5389,7 @@
         <v>1</v>
       </c>
       <c r="C150" s="1" t="s">
-        <v>498</v>
+        <v>488</v>
       </c>
       <c r="D150" s="1" t="s">
         <v>372</v>
@@ -5394,10 +5398,10 @@
         <v>40000</v>
       </c>
       <c r="F150" s="1" t="s">
-        <v>504</v>
+        <v>494</v>
       </c>
       <c r="G150" s="1" t="s">
-        <v>499</v>
+        <v>489</v>
       </c>
     </row>
     <row r="151" spans="1:7" ht="72" x14ac:dyDescent="0.3">
@@ -5408,7 +5412,7 @@
         <v>1</v>
       </c>
       <c r="C151" s="1" t="s">
-        <v>500</v>
+        <v>490</v>
       </c>
       <c r="D151" s="1" t="s">
         <v>366</v>
@@ -5417,10 +5421,10 @@
         <v>25000</v>
       </c>
       <c r="F151" s="1" t="s">
-        <v>503</v>
+        <v>493</v>
       </c>
       <c r="G151" s="1" t="s">
-        <v>501</v>
+        <v>491</v>
       </c>
     </row>
   </sheetData>

</xml_diff>